<commit_message>
chore(demo): V2 approval, prompt-lock file, HF negative-prompt support
- dashboard.xlsx: row 2 Approval Status -> Approved (V2 accepted)
- PROMPT.md: master consistency-lock file (character/outfit/camera/set/seed locks)
- scripts/hf_scene.py: --negative CLI arg for LTX negative prompting
</commit_message>
<xml_diff>
--- a/dashboard.xlsx
+++ b/dashboard.xlsx
@@ -552,32 +552,32 @@
       </c>
       <c r="G2" s="2" t="inlineStr">
         <is>
+          <t>Approved</t>
+        </is>
+      </c>
+      <c r="H2" s="2" t="inlineStr">
+        <is>
           <t>Pending</t>
         </is>
       </c>
-      <c r="H2" s="2" t="inlineStr">
+      <c r="I2" s="2" t="inlineStr">
         <is>
           <t>Pending</t>
         </is>
       </c>
-      <c r="I2" s="2" t="inlineStr">
+      <c r="J2" s="2" t="inlineStr">
         <is>
           <t>Pending</t>
         </is>
       </c>
-      <c r="J2" s="2" t="inlineStr">
-        <is>
-          <t>Pending</t>
-        </is>
-      </c>
       <c r="K2" s="2" t="inlineStr">
         <is>
-          <t>2026-09-30T14:37:33Z</t>
+          <t>2026-10-01T20:09:48Z</t>
         </is>
       </c>
       <c r="L2" s="2" t="inlineStr">
         <is>
-          <t>/home/hatch/workspace/AI-Social-Media-Content-Automation/storage/pending/2026-09-30-row2/final.mp4</t>
+          <t>/home/hatch/workspace/AI-Social-Media-Content-Automation/storage/pending/2026-10-01-row2-v2/final_v2.mp4</t>
         </is>
       </c>
       <c r="M2" s="3" t="inlineStr"/>

</xml_diff>